<commit_message>
Added the omitted species the complete adsorbate species were used for this generation
</commit_message>
<xml_diff>
--- a/Data/Cu3Sn0001/vibrational_freq_zpe_Cu3Sn0001.xlsx
+++ b/Data/Cu3Sn0001/vibrational_freq_zpe_Cu3Sn0001.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y29"/>
+  <dimension ref="A1:Y31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -934,206 +934,200 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>OCHCH2OHX</t>
+          <t>OCHCHX</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>3760.959902</v>
+        <v>3031.734648</v>
       </c>
       <c r="D11" t="n">
-        <v>2899.287586</v>
+        <v>2928.665324</v>
       </c>
       <c r="E11" t="n">
-        <v>2812.964825</v>
+        <v>1437.364468</v>
       </c>
       <c r="F11" t="n">
-        <v>2801.644158</v>
+        <v>1310.324008</v>
       </c>
       <c r="G11" t="n">
-        <v>1661.763666</v>
+        <v>1240.302447</v>
       </c>
       <c r="H11" t="n">
-        <v>1396.575053</v>
+        <v>1087.184672</v>
       </c>
       <c r="I11" t="n">
-        <v>1355.351409</v>
+        <v>913.592535</v>
       </c>
       <c r="J11" t="n">
-        <v>1317.314325</v>
+        <v>769.991254</v>
       </c>
       <c r="K11" t="n">
-        <v>1183.828124</v>
+        <v>677.418262</v>
       </c>
       <c r="L11" t="n">
-        <v>1182.713807</v>
+        <v>389.934159</v>
       </c>
       <c r="M11" t="n">
-        <v>1067.899716</v>
+        <v>306.072857</v>
       </c>
       <c r="N11" t="n">
-        <v>1039.142561</v>
+        <v>301.973462</v>
       </c>
       <c r="O11" t="n">
-        <v>991.713105</v>
+        <v>243.809634</v>
       </c>
       <c r="P11" t="n">
-        <v>670.974473</v>
+        <v>133.062055</v>
       </c>
       <c r="Q11" t="n">
-        <v>543.079268</v>
-      </c>
-      <c r="R11" t="n">
-        <v>326.244348</v>
-      </c>
-      <c r="S11" t="n">
-        <v>215.835917</v>
-      </c>
-      <c r="T11" t="n">
-        <v>193.145272</v>
-      </c>
-      <c r="U11" t="n">
-        <v>133.714635</v>
-      </c>
-      <c r="V11" t="n">
-        <v>97.166275</v>
-      </c>
-      <c r="W11" t="n">
-        <v>82.55182499999999</v>
-      </c>
-      <c r="X11" t="n">
-        <v>45.54051</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>21.71635</v>
-      </c>
+        <v>100.280389</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OCHCH2X</t>
+          <t>OCHCH2OHX</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>3186.086606</v>
+        <v>3760.959902</v>
       </c>
       <c r="D12" t="n">
-        <v>3081.758645</v>
+        <v>2899.287586</v>
       </c>
       <c r="E12" t="n">
-        <v>3040.467958</v>
+        <v>2812.964825</v>
       </c>
       <c r="F12" t="n">
-        <v>1605.342019</v>
+        <v>2801.644158</v>
       </c>
       <c r="G12" t="n">
-        <v>1363.471653</v>
+        <v>1661.763666</v>
       </c>
       <c r="H12" t="n">
-        <v>1289.279732</v>
+        <v>1396.575053</v>
       </c>
       <c r="I12" t="n">
-        <v>1127.958764</v>
+        <v>1355.351409</v>
       </c>
       <c r="J12" t="n">
-        <v>932.953389</v>
+        <v>1317.314325</v>
       </c>
       <c r="K12" t="n">
-        <v>930.328941</v>
+        <v>1183.828124</v>
       </c>
       <c r="L12" t="n">
-        <v>804.7278260000001</v>
+        <v>1182.713807</v>
       </c>
       <c r="M12" t="n">
-        <v>694.461248</v>
+        <v>1067.899716</v>
       </c>
       <c r="N12" t="n">
-        <v>530.086886</v>
+        <v>1039.142561</v>
       </c>
       <c r="O12" t="n">
-        <v>244.278357</v>
+        <v>991.713105</v>
       </c>
       <c r="P12" t="n">
-        <v>229.533854</v>
+        <v>670.974473</v>
       </c>
       <c r="Q12" t="n">
-        <v>159.72332</v>
+        <v>543.079268</v>
       </c>
       <c r="R12" t="n">
-        <v>119.151411</v>
+        <v>326.244348</v>
       </c>
       <c r="S12" t="n">
-        <v>46.736506</v>
-      </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
+        <v>215.835917</v>
+      </c>
+      <c r="T12" t="n">
+        <v>193.145272</v>
+      </c>
+      <c r="U12" t="n">
+        <v>133.714635</v>
+      </c>
+      <c r="V12" t="n">
+        <v>97.166275</v>
+      </c>
+      <c r="W12" t="n">
+        <v>82.55182499999999</v>
+      </c>
+      <c r="X12" t="n">
+        <v>45.54051</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>21.71635</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OCHCH3X</t>
+          <t>OCHCH2X</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>3077.479531</v>
+        <v>3186.086606</v>
       </c>
       <c r="D13" t="n">
-        <v>2988.193119</v>
+        <v>3081.758645</v>
       </c>
       <c r="E13" t="n">
-        <v>2934.783962</v>
+        <v>3040.467958</v>
       </c>
       <c r="F13" t="n">
-        <v>2886.151836</v>
+        <v>1605.342019</v>
       </c>
       <c r="G13" t="n">
-        <v>1659.583984</v>
+        <v>1363.471653</v>
       </c>
       <c r="H13" t="n">
-        <v>1405.59726</v>
+        <v>1289.279732</v>
       </c>
       <c r="I13" t="n">
-        <v>1389.906193</v>
+        <v>1127.958764</v>
       </c>
       <c r="J13" t="n">
-        <v>1371.869057</v>
+        <v>932.953389</v>
       </c>
       <c r="K13" t="n">
-        <v>1307.970574</v>
+        <v>930.328941</v>
       </c>
       <c r="L13" t="n">
-        <v>1084.550899</v>
+        <v>804.7278260000001</v>
       </c>
       <c r="M13" t="n">
-        <v>1060.781699</v>
+        <v>694.461248</v>
       </c>
       <c r="N13" t="n">
-        <v>932.15428</v>
+        <v>530.086886</v>
       </c>
       <c r="O13" t="n">
-        <v>691.1046229999999</v>
+        <v>244.278357</v>
       </c>
       <c r="P13" t="n">
-        <v>505.669144</v>
+        <v>229.533854</v>
       </c>
       <c r="Q13" t="n">
-        <v>158.322608</v>
+        <v>159.72332</v>
       </c>
       <c r="R13" t="n">
-        <v>122.434841</v>
+        <v>119.151411</v>
       </c>
       <c r="S13" t="n">
-        <v>84.06042100000001</v>
-      </c>
-      <c r="T13" t="n">
-        <v>52.811999</v>
-      </c>
+        <v>46.736506</v>
+      </c>
+      <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
@@ -1143,162 +1137,174 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OCH2CH3X</t>
+          <t>OCHCH3X</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
+        <v>3077.479531</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2988.193119</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2934.783962</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2886.151836</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1659.583984</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1405.59726</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1389.906193</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1371.869057</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1307.970574</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1084.550899</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1060.781699</v>
+      </c>
+      <c r="N14" t="n">
+        <v>932.15428</v>
+      </c>
+      <c r="O14" t="n">
+        <v>691.1046229999999</v>
+      </c>
+      <c r="P14" t="n">
+        <v>505.669144</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>158.322608</v>
+      </c>
+      <c r="R14" t="n">
+        <v>122.434841</v>
+      </c>
+      <c r="S14" t="n">
+        <v>84.06042100000001</v>
+      </c>
+      <c r="T14" t="n">
+        <v>52.811999</v>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OCH2CH3X</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="n">
         <v>3043.076341</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>3035.891821</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E15" t="n">
         <v>2978.487806</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F15" t="n">
         <v>2958.902071</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G15" t="n">
         <v>2941.129618</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H15" t="n">
         <v>1455.632619</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I15" t="n">
         <v>1433.698925</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J15" t="n">
         <v>1426.194657</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K15" t="n">
         <v>1350.071207</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L15" t="n">
         <v>1329.752985</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M15" t="n">
         <v>1253.445489</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N15" t="n">
         <v>1117.42644</v>
       </c>
-      <c r="O14" t="n">
+      <c r="O15" t="n">
         <v>1073.92053</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P15" t="n">
         <v>1007.715437</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q15" t="n">
         <v>854.979912</v>
       </c>
-      <c r="R14" t="n">
+      <c r="R15" t="n">
         <v>773.964298</v>
       </c>
-      <c r="S14" t="n">
+      <c r="S15" t="n">
         <v>460.484287</v>
       </c>
-      <c r="T14" t="n">
+      <c r="T15" t="n">
         <v>301.008865</v>
       </c>
-      <c r="U14" t="n">
+      <c r="U15" t="n">
         <v>252.217327</v>
       </c>
-      <c r="V14" t="n">
+      <c r="V15" t="n">
         <v>217.96169</v>
       </c>
-      <c r="W14" t="n">
+      <c r="W15" t="n">
         <v>173.881887</v>
       </c>
-      <c r="X14" t="n">
+      <c r="X15" t="n">
         <v>81.064375</v>
       </c>
-      <c r="Y14" t="n">
+      <c r="Y15" t="n">
         <v>36.887899</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>molecule</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>vib freq (meV)</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COOHX</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="n">
-        <v>433.340273</v>
-      </c>
-      <c r="D18" t="n">
-        <v>181.316394</v>
-      </c>
-      <c r="E18" t="n">
-        <v>154.73463</v>
-      </c>
-      <c r="F18" t="n">
-        <v>134.223874</v>
-      </c>
-      <c r="G18" t="n">
-        <v>84.54969199999999</v>
-      </c>
-      <c r="H18" t="n">
-        <v>80.95805900000001</v>
-      </c>
-      <c r="I18" t="n">
-        <v>49.027124</v>
-      </c>
-      <c r="J18" t="n">
-        <v>33.137685</v>
-      </c>
-      <c r="K18" t="n">
-        <v>27.233749</v>
-      </c>
-      <c r="L18" t="n">
-        <v>15.430965</v>
-      </c>
-      <c r="M18" t="n">
-        <v>13.972942</v>
-      </c>
-      <c r="N18" t="n">
-        <v>6.294202</v>
-      </c>
+          <t>molecule</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>vib freq (meV)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
@@ -1314,45 +1320,45 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OCHOX</t>
+          <t>COOHX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>364.069163</v>
+        <v>433.340273</v>
       </c>
       <c r="D19" t="n">
-        <v>189.951535</v>
+        <v>181.316394</v>
       </c>
       <c r="E19" t="n">
-        <v>164.358397</v>
+        <v>154.73463</v>
       </c>
       <c r="F19" t="n">
-        <v>162.697554</v>
+        <v>134.223874</v>
       </c>
       <c r="G19" t="n">
-        <v>121.406894</v>
+        <v>84.54969199999999</v>
       </c>
       <c r="H19" t="n">
-        <v>90.756736</v>
+        <v>80.95805900000001</v>
       </c>
       <c r="I19" t="n">
-        <v>36.552445</v>
+        <v>49.027124</v>
       </c>
       <c r="J19" t="n">
-        <v>36.244812</v>
+        <v>33.137685</v>
       </c>
       <c r="K19" t="n">
-        <v>33.598119</v>
+        <v>27.233749</v>
       </c>
       <c r="L19" t="n">
-        <v>11.672094</v>
+        <v>15.430965</v>
       </c>
       <c r="M19" t="n">
-        <v>11.478283</v>
+        <v>13.972942</v>
       </c>
       <c r="N19" t="n">
-        <v>8.5329</v>
+        <v>6.294202</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
@@ -1369,34 +1375,46 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>COX</t>
+          <t>OCHOX</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>249.428503</v>
+        <v>364.069163</v>
       </c>
       <c r="D20" t="n">
-        <v>41.375594</v>
+        <v>189.951535</v>
       </c>
       <c r="E20" t="n">
-        <v>39.43894</v>
+        <v>164.358397</v>
       </c>
       <c r="F20" t="n">
-        <v>34.975385</v>
+        <v>162.697554</v>
       </c>
       <c r="G20" t="n">
-        <v>8.0144</v>
+        <v>121.406894</v>
       </c>
       <c r="H20" t="n">
-        <v>4.8843</v>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+        <v>90.756736</v>
+      </c>
+      <c r="I20" t="n">
+        <v>36.552445</v>
+      </c>
+      <c r="J20" t="n">
+        <v>36.244812</v>
+      </c>
+      <c r="K20" t="n">
+        <v>33.598119</v>
+      </c>
+      <c r="L20" t="n">
+        <v>11.672094</v>
+      </c>
+      <c r="M20" t="n">
+        <v>11.478283</v>
+      </c>
+      <c r="N20" t="n">
+        <v>8.5329</v>
+      </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
@@ -1412,46 +1430,34 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OCCOX</t>
+          <t>COX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>196.505879</v>
+        <v>249.428503</v>
       </c>
       <c r="D21" t="n">
-        <v>190.726891</v>
+        <v>41.375594</v>
       </c>
       <c r="E21" t="n">
-        <v>83.829748</v>
+        <v>39.43894</v>
       </c>
       <c r="F21" t="n">
-        <v>82.16173000000001</v>
+        <v>34.975385</v>
       </c>
       <c r="G21" t="n">
-        <v>56.692166</v>
+        <v>8.0144</v>
       </c>
       <c r="H21" t="n">
-        <v>43.922241</v>
-      </c>
-      <c r="I21" t="n">
-        <v>37.991232</v>
-      </c>
-      <c r="J21" t="n">
-        <v>34.597855</v>
-      </c>
-      <c r="K21" t="n">
-        <v>30.739072</v>
-      </c>
-      <c r="L21" t="n">
-        <v>24.502418</v>
-      </c>
-      <c r="M21" t="n">
-        <v>14.347112</v>
-      </c>
-      <c r="N21" t="n">
-        <v>11.2294</v>
-      </c>
+        <v>4.8843</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
@@ -1467,40 +1473,46 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CHOX</t>
+          <t>OCCOX</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>345.391922</v>
+        <v>196.505879</v>
       </c>
       <c r="D22" t="n">
-        <v>183.337231</v>
+        <v>190.726891</v>
       </c>
       <c r="E22" t="n">
-        <v>154.928533</v>
+        <v>83.829748</v>
       </c>
       <c r="F22" t="n">
-        <v>87.449752</v>
+        <v>82.16173000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>58.228871</v>
+        <v>56.692166</v>
       </c>
       <c r="H22" t="n">
-        <v>32.70526</v>
+        <v>43.922241</v>
       </c>
       <c r="I22" t="n">
-        <v>25.887826</v>
+        <v>37.991232</v>
       </c>
       <c r="J22" t="n">
-        <v>16.858711</v>
+        <v>34.597855</v>
       </c>
       <c r="K22" t="n">
-        <v>12.203669</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
+        <v>30.739072</v>
+      </c>
+      <c r="L22" t="n">
+        <v>24.502418</v>
+      </c>
+      <c r="M22" t="n">
+        <v>14.347112</v>
+      </c>
+      <c r="N22" t="n">
+        <v>11.2294</v>
+      </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
@@ -1516,52 +1528,42 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>COCHOX</t>
+          <t>CHOX</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>344.554589</v>
+        <v>345.391922</v>
       </c>
       <c r="D23" t="n">
-        <v>206.600301</v>
+        <v>183.337231</v>
       </c>
       <c r="E23" t="n">
-        <v>185.959084</v>
+        <v>154.928533</v>
       </c>
       <c r="F23" t="n">
-        <v>160.591808</v>
+        <v>87.449752</v>
       </c>
       <c r="G23" t="n">
-        <v>112.374194</v>
+        <v>58.228871</v>
       </c>
       <c r="H23" t="n">
-        <v>106.610396</v>
+        <v>32.70526</v>
       </c>
       <c r="I23" t="n">
-        <v>79.29728</v>
+        <v>25.887826</v>
       </c>
       <c r="J23" t="n">
-        <v>52.22682</v>
+        <v>16.858711</v>
       </c>
       <c r="K23" t="n">
-        <v>34.385467</v>
-      </c>
-      <c r="L23" t="n">
-        <v>30.347449</v>
-      </c>
-      <c r="M23" t="n">
-        <v>22.100583</v>
-      </c>
-      <c r="N23" t="n">
-        <v>12.86552</v>
-      </c>
-      <c r="O23" t="n">
-        <v>10.276664</v>
-      </c>
-      <c r="P23" t="n">
-        <v>5.580615</v>
-      </c>
+        <v>12.203669</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
@@ -1575,64 +1577,56 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>OCHOCHX</t>
+          <t>COCHOX</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>378.42007</v>
+        <v>344.554589</v>
       </c>
       <c r="D24" t="n">
-        <v>373.387887</v>
+        <v>206.600301</v>
       </c>
       <c r="E24" t="n">
-        <v>178.207461</v>
+        <v>185.959084</v>
       </c>
       <c r="F24" t="n">
-        <v>171.212661</v>
+        <v>160.591808</v>
       </c>
       <c r="G24" t="n">
-        <v>156.267143</v>
+        <v>112.374194</v>
       </c>
       <c r="H24" t="n">
-        <v>146.326166</v>
+        <v>106.610396</v>
       </c>
       <c r="I24" t="n">
-        <v>123.484492</v>
+        <v>79.29728</v>
       </c>
       <c r="J24" t="n">
-        <v>106.1993</v>
+        <v>52.22682</v>
       </c>
       <c r="K24" t="n">
-        <v>97.92911100000001</v>
+        <v>34.385467</v>
       </c>
       <c r="L24" t="n">
-        <v>85.231391</v>
+        <v>30.347449</v>
       </c>
       <c r="M24" t="n">
-        <v>58.086738</v>
+        <v>22.100583</v>
       </c>
       <c r="N24" t="n">
-        <v>44.300061</v>
+        <v>12.86552</v>
       </c>
       <c r="O24" t="n">
-        <v>30.240953</v>
+        <v>10.276664</v>
       </c>
       <c r="P24" t="n">
-        <v>29.600096</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>22.669397</v>
-      </c>
-      <c r="R24" t="n">
-        <v>11.034587</v>
-      </c>
-      <c r="S24" t="n">
-        <v>7.60708</v>
-      </c>
-      <c r="T24" t="n">
-        <v>6.86155</v>
-      </c>
+        <v>5.580615</v>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
@@ -1642,211 +1636,197 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>OCHCHOHX</t>
+          <t>OCHOCHX</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>469.239344</v>
+        <v>378.42007</v>
       </c>
       <c r="D25" t="n">
-        <v>382.34295</v>
+        <v>373.387887</v>
       </c>
       <c r="E25" t="n">
-        <v>378.448916</v>
+        <v>178.207461</v>
       </c>
       <c r="F25" t="n">
-        <v>204.175575</v>
+        <v>171.212661</v>
       </c>
       <c r="G25" t="n">
-        <v>161.908549</v>
+        <v>156.267143</v>
       </c>
       <c r="H25" t="n">
-        <v>158.407489</v>
+        <v>146.326166</v>
       </c>
       <c r="I25" t="n">
-        <v>146.668122</v>
+        <v>123.484492</v>
       </c>
       <c r="J25" t="n">
-        <v>140.44097</v>
+        <v>106.1993</v>
       </c>
       <c r="K25" t="n">
-        <v>133.497185</v>
+        <v>97.92911100000001</v>
       </c>
       <c r="L25" t="n">
-        <v>104.785551</v>
+        <v>85.231391</v>
       </c>
       <c r="M25" t="n">
-        <v>95.841633</v>
+        <v>58.086738</v>
       </c>
       <c r="N25" t="n">
-        <v>73.27364</v>
+        <v>44.300061</v>
       </c>
       <c r="O25" t="n">
-        <v>47.72484</v>
+        <v>30.240953</v>
       </c>
       <c r="P25" t="n">
-        <v>45.334407</v>
+        <v>29.600096</v>
       </c>
       <c r="Q25" t="n">
-        <v>27.072714</v>
+        <v>22.669397</v>
       </c>
       <c r="R25" t="n">
-        <v>26.113098</v>
+        <v>11.034587</v>
       </c>
       <c r="S25" t="n">
-        <v>18.222911</v>
+        <v>7.60708</v>
       </c>
       <c r="T25" t="n">
-        <v>17.009777</v>
-      </c>
-      <c r="U25" t="n">
-        <v>14.87267</v>
-      </c>
-      <c r="V25" t="n">
-        <v>9.24502</v>
-      </c>
-      <c r="W25" t="n">
-        <v>3.065948</v>
-      </c>
+        <v>6.86155</v>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OCHCH2OHX</t>
+          <t>OCHCHOHX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>466.299389</v>
+        <v>469.239344</v>
       </c>
       <c r="D26" t="n">
-        <v>359.465685</v>
+        <v>382.34295</v>
       </c>
       <c r="E26" t="n">
-        <v>348.763032</v>
+        <v>378.448916</v>
       </c>
       <c r="F26" t="n">
-        <v>347.359449</v>
+        <v>204.175575</v>
       </c>
       <c r="G26" t="n">
-        <v>206.032343</v>
+        <v>161.908549</v>
       </c>
       <c r="H26" t="n">
-        <v>173.15316</v>
+        <v>158.407489</v>
       </c>
       <c r="I26" t="n">
-        <v>168.042082</v>
+        <v>146.668122</v>
       </c>
       <c r="J26" t="n">
-        <v>163.326087</v>
+        <v>140.44097</v>
       </c>
       <c r="K26" t="n">
-        <v>146.775915</v>
+        <v>133.497185</v>
       </c>
       <c r="L26" t="n">
-        <v>146.637757</v>
+        <v>104.785551</v>
       </c>
       <c r="M26" t="n">
-        <v>132.402631</v>
+        <v>95.841633</v>
       </c>
       <c r="N26" t="n">
-        <v>128.837199</v>
+        <v>73.27364</v>
       </c>
       <c r="O26" t="n">
-        <v>122.956699</v>
+        <v>47.72484</v>
       </c>
       <c r="P26" t="n">
-        <v>83.190195</v>
+        <v>45.334407</v>
       </c>
       <c r="Q26" t="n">
-        <v>67.333217</v>
+        <v>27.072714</v>
       </c>
       <c r="R26" t="n">
-        <v>40.449126</v>
+        <v>26.113098</v>
       </c>
       <c r="S26" t="n">
-        <v>26.760231</v>
+        <v>18.222911</v>
       </c>
       <c r="T26" t="n">
-        <v>23.946951</v>
+        <v>17.009777</v>
       </c>
       <c r="U26" t="n">
-        <v>16.578494</v>
+        <v>14.87267</v>
       </c>
       <c r="V26" t="n">
-        <v>12.047077</v>
+        <v>9.24502</v>
       </c>
       <c r="W26" t="n">
-        <v>10.235117</v>
-      </c>
-      <c r="X26" t="n">
-        <v>5.646301</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>2.692483</v>
-      </c>
+        <v>3.065948</v>
+      </c>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OCHCH2X</t>
+          <t>OCHCHX</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>395.024216</v>
+        <v>375.887021</v>
       </c>
       <c r="D27" t="n">
-        <v>382.089203</v>
+        <v>363.108059</v>
       </c>
       <c r="E27" t="n">
-        <v>376.969813</v>
+        <v>178.210401</v>
       </c>
       <c r="F27" t="n">
-        <v>199.036954</v>
+        <v>162.459399</v>
       </c>
       <c r="G27" t="n">
-        <v>169.048864</v>
+        <v>153.777835</v>
       </c>
       <c r="H27" t="n">
-        <v>159.850242</v>
+        <v>134.793659</v>
       </c>
       <c r="I27" t="n">
-        <v>139.849</v>
+        <v>113.270987</v>
       </c>
       <c r="J27" t="n">
-        <v>115.671426</v>
+        <v>95.466705</v>
       </c>
       <c r="K27" t="n">
-        <v>115.346036</v>
+        <v>83.98912199999999</v>
       </c>
       <c r="L27" t="n">
-        <v>99.773489</v>
+        <v>48.345652</v>
       </c>
       <c r="M27" t="n">
-        <v>86.102182</v>
+        <v>37.948181</v>
       </c>
       <c r="N27" t="n">
-        <v>65.722368</v>
+        <v>37.439921</v>
       </c>
       <c r="O27" t="n">
-        <v>30.286643</v>
+        <v>30.228528</v>
       </c>
       <c r="P27" t="n">
-        <v>28.458558</v>
+        <v>16.497585</v>
       </c>
       <c r="Q27" t="n">
-        <v>19.803159</v>
-      </c>
-      <c r="R27" t="n">
-        <v>14.772886</v>
-      </c>
-      <c r="S27" t="n">
-        <v>5.794586</v>
-      </c>
+        <v>12.433178</v>
+      </c>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
@@ -1857,144 +1837,286 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OCHCH3X</t>
+          <t>OCHCH2OHX</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>381.558661</v>
+        <v>466.299389</v>
       </c>
       <c r="D28" t="n">
-        <v>370.488562</v>
+        <v>359.465685</v>
       </c>
       <c r="E28" t="n">
-        <v>363.866673</v>
+        <v>348.763032</v>
       </c>
       <c r="F28" t="n">
-        <v>357.837061</v>
+        <v>347.359449</v>
       </c>
       <c r="G28" t="n">
-        <v>205.762097</v>
+        <v>206.032343</v>
       </c>
       <c r="H28" t="n">
-        <v>174.271771</v>
+        <v>173.15316</v>
       </c>
       <c r="I28" t="n">
-        <v>172.326328</v>
+        <v>168.042082</v>
       </c>
       <c r="J28" t="n">
-        <v>170.090009</v>
+        <v>163.326087</v>
       </c>
       <c r="K28" t="n">
-        <v>162.16761</v>
+        <v>146.775915</v>
       </c>
       <c r="L28" t="n">
-        <v>134.467113</v>
+        <v>146.637757</v>
       </c>
       <c r="M28" t="n">
-        <v>131.520109</v>
+        <v>132.402631</v>
       </c>
       <c r="N28" t="n">
-        <v>115.572349</v>
+        <v>128.837199</v>
       </c>
       <c r="O28" t="n">
-        <v>85.686014</v>
+        <v>122.956699</v>
       </c>
       <c r="P28" t="n">
-        <v>62.694955</v>
+        <v>83.190195</v>
       </c>
       <c r="Q28" t="n">
-        <v>19.629493</v>
+        <v>67.333217</v>
       </c>
       <c r="R28" t="n">
-        <v>15.179979</v>
+        <v>40.449126</v>
       </c>
       <c r="S28" t="n">
-        <v>10.422159</v>
+        <v>26.760231</v>
       </c>
       <c r="T28" t="n">
-        <v>6.54785</v>
-      </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
+        <v>23.946951</v>
+      </c>
+      <c r="U28" t="n">
+        <v>16.578494</v>
+      </c>
+      <c r="V28" t="n">
+        <v>12.047077</v>
+      </c>
+      <c r="W28" t="n">
+        <v>10.235117</v>
+      </c>
+      <c r="X28" t="n">
+        <v>5.646301</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>2.692483</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OCH2CH3X</t>
+          <t>OCHCH2X</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
+        <v>395.024216</v>
+      </c>
+      <c r="D29" t="n">
+        <v>382.089203</v>
+      </c>
+      <c r="E29" t="n">
+        <v>376.969813</v>
+      </c>
+      <c r="F29" t="n">
+        <v>199.036954</v>
+      </c>
+      <c r="G29" t="n">
+        <v>169.048864</v>
+      </c>
+      <c r="H29" t="n">
+        <v>159.850242</v>
+      </c>
+      <c r="I29" t="n">
+        <v>139.849</v>
+      </c>
+      <c r="J29" t="n">
+        <v>115.671426</v>
+      </c>
+      <c r="K29" t="n">
+        <v>115.346036</v>
+      </c>
+      <c r="L29" t="n">
+        <v>99.773489</v>
+      </c>
+      <c r="M29" t="n">
+        <v>86.102182</v>
+      </c>
+      <c r="N29" t="n">
+        <v>65.722368</v>
+      </c>
+      <c r="O29" t="n">
+        <v>30.286643</v>
+      </c>
+      <c r="P29" t="n">
+        <v>28.458558</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>19.803159</v>
+      </c>
+      <c r="R29" t="n">
+        <v>14.772886</v>
+      </c>
+      <c r="S29" t="n">
+        <v>5.794586</v>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>OCHCH3X</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="n">
+        <v>381.558661</v>
+      </c>
+      <c r="D30" t="n">
+        <v>370.488562</v>
+      </c>
+      <c r="E30" t="n">
+        <v>363.866673</v>
+      </c>
+      <c r="F30" t="n">
+        <v>357.837061</v>
+      </c>
+      <c r="G30" t="n">
+        <v>205.762097</v>
+      </c>
+      <c r="H30" t="n">
+        <v>174.271771</v>
+      </c>
+      <c r="I30" t="n">
+        <v>172.326328</v>
+      </c>
+      <c r="J30" t="n">
+        <v>170.090009</v>
+      </c>
+      <c r="K30" t="n">
+        <v>162.16761</v>
+      </c>
+      <c r="L30" t="n">
+        <v>134.467113</v>
+      </c>
+      <c r="M30" t="n">
+        <v>131.520109</v>
+      </c>
+      <c r="N30" t="n">
+        <v>115.572349</v>
+      </c>
+      <c r="O30" t="n">
+        <v>85.686014</v>
+      </c>
+      <c r="P30" t="n">
+        <v>62.694955</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>19.629493</v>
+      </c>
+      <c r="R30" t="n">
+        <v>15.179979</v>
+      </c>
+      <c r="S30" t="n">
+        <v>10.422159</v>
+      </c>
+      <c r="T30" t="n">
+        <v>6.54785</v>
+      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>OCH2CH3X</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="n">
         <v>377.293211</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D31" t="n">
         <v>376.402444</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E31" t="n">
         <v>369.285257</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F31" t="n">
         <v>366.856936</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G31" t="n">
         <v>364.653434</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H31" t="n">
         <v>180.475362</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I31" t="n">
         <v>177.755932</v>
       </c>
-      <c r="J29" t="n">
+      <c r="J31" t="n">
         <v>176.825522</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K31" t="n">
         <v>167.387421</v>
       </c>
-      <c r="L29" t="n">
+      <c r="L31" t="n">
         <v>164.868284</v>
       </c>
-      <c r="M29" t="n">
+      <c r="M31" t="n">
         <v>155.407364</v>
       </c>
-      <c r="N29" t="n">
+      <c r="N31" t="n">
         <v>138.543159</v>
       </c>
-      <c r="O29" t="n">
+      <c r="O31" t="n">
         <v>133.149116</v>
       </c>
-      <c r="P29" t="n">
+      <c r="P31" t="n">
         <v>124.940734</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="Q31" t="n">
         <v>106.003951</v>
       </c>
-      <c r="R29" t="n">
+      <c r="R31" t="n">
         <v>95.9593</v>
       </c>
-      <c r="S29" t="n">
+      <c r="S31" t="n">
         <v>57.092749</v>
       </c>
-      <c r="T29" t="n">
+      <c r="T31" t="n">
         <v>37.320326</v>
       </c>
-      <c r="U29" t="n">
+      <c r="U31" t="n">
         <v>31.270949</v>
       </c>
-      <c r="V29" t="n">
+      <c r="V31" t="n">
         <v>27.023793</v>
       </c>
-      <c r="W29" t="n">
+      <c r="W31" t="n">
         <v>21.558597</v>
       </c>
-      <c r="X29" t="n">
+      <c r="X31" t="n">
         <v>10.050697</v>
       </c>
-      <c r="Y29" t="n">
+      <c r="Y31" t="n">
         <v>4.573515</v>
       </c>
     </row>
@@ -2009,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2120,44 +2242,55 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>OCHCH2OHX</t>
+          <t>OCHCHX</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>1.599471</v>
+        <v>0.921932</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>OCHCH2X</t>
+          <t>OCHCH2OHX</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>1.201804</v>
+        <v>1.599471</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OCHCH3X</t>
+          <t>OCHCH2X</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>1.47005</v>
+        <v>1.201804</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OCH2CH3X</t>
+          <t>OCHCH3X</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
+        <v>1.47005</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OCH2CH3X</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="n">
         <v>1.832356</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added the missing frequency the complete frequency data was used to re-generate the thermodata
</commit_message>
<xml_diff>
--- a/Data/Cu3Sn0001/vibrational_freq_zpe_Cu3Sn0001.xlsx
+++ b/Data/Cu3Sn0001/vibrational_freq_zpe_Cu3Sn0001.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y31"/>
+  <dimension ref="A1:Z31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,7 @@
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -529,6 +530,7 @@
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -584,6 +586,7 @@
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -627,6 +630,7 @@
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -682,6 +686,7 @@
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -731,6 +736,7 @@
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -781,7 +787,9 @@
       <c r="P8" t="n">
         <v>45.010719</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
+      <c r="Q8" t="n">
+        <v>17.010043</v>
+      </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
@@ -790,6 +798,7 @@
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -857,6 +866,7 @@
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -930,6 +940,7 @@
       </c>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -991,6 +1002,7 @@
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1068,6 +1080,9 @@
       <c r="Y12" t="n">
         <v>21.71635</v>
       </c>
+      <c r="Z12" t="n">
+        <v>29.811134</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1127,12 +1142,15 @@
       <c r="S13" t="n">
         <v>46.736506</v>
       </c>
-      <c r="T13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>34.79086</v>
+      </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1195,11 +1213,18 @@
       <c r="T14" t="n">
         <v>52.811999</v>
       </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>31.853387</v>
+      </c>
+      <c r="V14" t="n">
+        <v>54.802001</v>
+      </c>
+      <c r="W14" t="n">
+        <v>70.239797</v>
+      </c>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1276,6 +1301,9 @@
       </c>
       <c r="Y15" t="n">
         <v>36.887899</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>79.688348</v>
       </c>
     </row>
     <row r="18">
@@ -1316,6 +1344,7 @@
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1371,6 +1400,7 @@
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1426,6 +1456,7 @@
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1469,6 +1500,7 @@
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1524,6 +1556,7 @@
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1573,6 +1606,7 @@
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1623,7 +1657,9 @@
       <c r="P24" t="n">
         <v>5.580615</v>
       </c>
-      <c r="Q24" t="inlineStr"/>
+      <c r="Q24" t="n">
+        <v>2.108976</v>
+      </c>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
@@ -1632,6 +1668,7 @@
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1699,6 +1736,7 @@
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1772,6 +1810,7 @@
       </c>
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1833,6 +1872,7 @@
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1910,6 +1950,9 @@
       <c r="Y28" t="n">
         <v>2.692483</v>
       </c>
+      <c r="Z28" t="n">
+        <v>3.696108</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1969,12 +2012,15 @@
       <c r="S29" t="n">
         <v>5.794586</v>
       </c>
-      <c r="T29" t="inlineStr"/>
+      <c r="T29" t="n">
+        <v>4.313515</v>
+      </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2037,11 +2083,18 @@
       <c r="T30" t="n">
         <v>6.54785</v>
       </c>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
+      <c r="U30" t="n">
+        <v>3.949315</v>
+      </c>
+      <c r="V30" t="n">
+        <v>6.794579</v>
+      </c>
+      <c r="W30" t="n">
+        <v>8.708621000000001</v>
+      </c>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2118,6 +2171,9 @@
       </c>
       <c r="Y31" t="n">
         <v>4.573515</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>9.880091</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
OCCOX labeling changed changed the labeling to XCOXCO in RMG format
</commit_message>
<xml_diff>
--- a/Data/Cu3Sn0001/vibrational_freq_zpe_Cu3Sn0001.xlsx
+++ b/Data/Cu3Sn0001/vibrational_freq_zpe_Cu3Sn0001.xlsx
@@ -635,7 +635,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>OCCOX</t>
+          <t>XCOXCO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -1505,7 +1505,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OCCOX</t>
+          <t>XCOXCO</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OCCOX</t>
+          <t>XCOXCO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>

</xml_diff>